<commit_message>
Revert "db sync pull req"
</commit_message>
<xml_diff>
--- a/News_Dashboard/data/raw_news_database_Mondee.xlsx
+++ b/News_Dashboard/data/raw_news_database_Mondee.xlsx
@@ -2765,17 +2765,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Market conditions are currently stable.</t>
+          <t>Conduct a rapid feature gap analysis of Expedia's new back-office API and prioritize development of comparable or superior APIs within MONDEE's platform, targeting a 30‑day sprint to close the gap.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>No high-priority competitor moves detected in this timeframe.</t>
+          <t>Launch a targeted marketing campaign that showcases MONDEE's existing back-office tools and upcoming enhancements, positioning the brand as a more integrated solution for travel operators.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Continue tracking standard sector intelligence.</t>
+          <t>Pursue a strategic partnership with a specialized back-office software provider to bundle complementary tools, enabling MONDEE to offer a comprehensive suite faster than competitors.</t>
         </is>
       </c>
     </row>
@@ -2819,17 +2819,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>No competitor product launches or API releases cataloged.</t>
+          <t>Accelerate the development of a back‑office API that offers real‑time inventory and booking management, and release a beta version to our top 10 agency partners within 30 days to directly compete with Expedia TAAP’s new tools.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Digital feature velocity remains normal.</t>
+          <t>Initiate a joint integration pilot with Expedia TAAP to demonstrate seamless interoperability, positioning MONDEE as the preferred partner for agencies that use both platforms and highlighting our unique data‑driven insights.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Continue monitoring competitor release notes.</t>
+          <t>Launch a targeted marketing campaign that showcases MONDEE’s existing back‑office automation features—such as faster processing times and lower costs—positioning them as superior to Expedia’s newly released tools for travel agencies seeking efficiency.</t>
         </is>
       </c>
     </row>
@@ -2846,17 +2846,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Launch a dedicated back‑office API suite for travel advisors that mirrors Expedia TAAP’s features, prioritizing real‑time inventory, booking reference tools, and workflow automation to attract agencies seeking a seamless tech stack.</t>
+          <t>Develop and launch a back‑office API suite for travel advisors, mirroring Expedia TAAP’s new tools, and promote it through targeted webinars to capture agency demand.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Develop a white‑label travel engine similar to Priceline Partner Network, enabling partners to brand and sell curated itineraries while integrating with MONDEE’s core platform, thereby expanding our partner ecosystem.</t>
+          <t>Create a Vancouver‑centric travel bundle that highlights the new car‑free Granville Street, using MONDEE’s data to offer exclusive itineraries and partner with local businesses for cross‑promotions.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Create a Vancouver‑centric travel package API that highlights the new pedestrian zone, offering curated walking tours and local experiences, and promote it to travel agencies to capitalize on the city’s increased foot traffic.</t>
+          <t>Integrate MONDEE’s booking engine with Priceline Partner Network’s white‑label platform to provide agencies with a seamless, branded experience, and negotiate revenue‑share terms to expand market reach.</t>
         </is>
       </c>
     </row>
@@ -2900,17 +2900,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Develop a dedicated back-office API suite for travel advisors, mirroring Expedia TAAP's features, and partner with a major agency network to pilot it within 90 days.</t>
+          <t>Develop and launch a dedicated back‑office API suite for travel advisors, mirroring Expedia TAAP’s new tools, and offer a sandbox for agencies to integrate and test, positioning MONDEE as the go‑to platform for agency automation. Prioritize API documentation and developer support to accelerate adoption among mid‑size agencies.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Leverage our existing white-label engine to create a co-branded travel platform for a mid-sized agency, offering integrated booking and analytics, to compete with Priceline Partner Network's quiet engine.</t>
+          <t>Introduce a white‑label travel engine similar to Priceline Partner Network, enabling partners to brand and customize the booking experience, and target niche verticals such as corporate travel or experiential tours. Leverage existing data feeds to provide real‑time inventory and pricing, ensuring partners can compete with larger platforms.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Launch a targeted marketing campaign highlighting MONDEE's real-time data insights and AI-driven pricing tools, positioning us as the most efficient alternative to Expedia TAAP's new tools, and schedule a webinar for advisors within 30 days.</t>
+          <t>Collaborate with key travel advisors to pilot a new advisor‑centric feature set, including real‑time booking reference tools and workflow automation, and use the pilot data to refine the product roadmap. Publish case studies from early adopters to demonstrate ROI and attract additional agency clients.</t>
         </is>
       </c>
     </row>
@@ -2927,17 +2927,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Develop a dedicated back‑office API for travel advisors that includes real‑time inventory, commission tracking, and automated booking reference generation, directly addressing Expedia TAAP’s new toolset and positioning MONDEE as the preferred tech partner for agencies.</t>
+          <t>Launch a back‑office API suite for travel advisors that integrates booking, inventory, and commission management, mirroring Expedia TAAP, to retain agency partners and differentiate MONDEE’s platform. Develop a modular, developer‑friendly SDK that allows agencies to embed MONDEE’s core booking engine into their own portals within 90 days.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Launch a city‑partner program that provides travel advisors with a specialized API for pedestrian‑zone itineraries, using Vancouver’s Granville Street expansion as a pilot to showcase sustainable travel solutions and differentiate MONDEE’s offerings.</t>
+          <t>Partner with Vancouver city authorities to create a digital concierge service for the new Granville Street pedestrian zone, offering real‑time navigation, local business promotions, and exclusive offers to capture the increased foot traffic. Deploy a mobile app that aggregates local events, dining, and transport options, positioning MONDEE as the go‑to platform for downtown travelers.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Create a white‑label travel engine similar to Priceline Partner Network’s model, and secure exclusive distribution agreements with mid‑market agencies to capture the growing demand for customizable booking platforms.</t>
+          <t>Build a white‑label travel engine similar to Priceline Partner Network, enabling third‑party agencies to brand MONDEE’s booking infrastructure and expand revenue streams. Offer a revenue‑share model and dedicated support to attract agencies looking to launch their own branded travel portals within 6 months.</t>
         </is>
       </c>
     </row>
@@ -2981,17 +2981,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Develop and launch a back‑office API suite for travel advisors that includes booking reference generation and real‑time inventory access, mirroring Expedia TAAP’s new tools, and offer it as a free pilot to top 50 agencies.</t>
+          <t>Launch a dedicated back‑office API and suite of tools for travel advisors, mirroring Expedia TAAP’s offerings, and open a beta program for agencies to test and provide feedback.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Introduce a rewards program for travel advisors that rewards higher booking volumes, directly competing with Expedia TAAP’s rewards, and integrate it into the API so advisors can track points in real time.</t>
+          <t>Form a strategic partnership with a leading travel agency network to embed MONDEE’s white‑label engine, positioning it as a direct competitor to Priceline Partner Network’s platform.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Partner with a white‑label travel engine provider (e.g., Priceline Partner Network) to quickly roll out a customizable booking engine for agencies, positioning MONDEE as a one‑stop solution for agencies seeking both front‑end and back‑office capabilities.</t>
+          <t>Introduce a rewards program for advisors who book through MONDEE, offering tiered incentives and exclusive benefits to drive adoption and loyalty, similar to Expedia TAAP Rewards.</t>
         </is>
       </c>
     </row>

</xml_diff>